<commit_message>
- remove "Style" column from wallpaper_template.xlsx due to Wayfair's changes.
</commit_message>
<xml_diff>
--- a/assets/wallpaper_template.xlsx
+++ b/assets/wallpaper_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10830"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danielkravchenko/PycharmProjects/WayfairFlatMaker/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB921174-1D7F-1741-919F-229FCBDB288D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2173070D-2EBC-8749-B7A2-ABC243D471EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
     <author>Author</author>
   </authors>
   <commentList>
-    <comment ref="BX3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
+    <comment ref="BW3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
       <text>
         <r>
           <rPr>
@@ -64,7 +64,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BY3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000002000000}">
+    <comment ref="BX3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000002000000}">
       <text>
         <r>
           <rPr>
@@ -77,7 +77,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BZ3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000003000000}">
+    <comment ref="BY3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000003000000}">
       <text>
         <r>
           <rPr>
@@ -90,7 +90,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CA3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000004000000}">
+    <comment ref="BZ3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000004000000}">
       <text>
         <r>
           <rPr>
@@ -103,7 +103,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CG3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000005000000}">
+    <comment ref="CF3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000005000000}">
       <text>
         <r>
           <rPr>
@@ -116,7 +116,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CH3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000006000000}">
+    <comment ref="CG3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000006000000}">
       <text>
         <r>
           <rPr>
@@ -129,7 +129,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CK3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000007000000}">
+    <comment ref="CJ3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000007000000}">
       <text>
         <r>
           <rPr>
@@ -142,7 +142,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CL3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000008000000}">
+    <comment ref="CK3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000008000000}">
       <text>
         <r>
           <rPr>
@@ -155,7 +155,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CO3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000009000000}">
+    <comment ref="CN3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000009000000}">
       <text>
         <r>
           <rPr>
@@ -168,7 +168,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CP3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000A000000}">
+    <comment ref="CO3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000A000000}">
       <text>
         <r>
           <rPr>
@@ -181,7 +181,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CW3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000B000000}">
+    <comment ref="CV3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000B000000}">
       <text>
         <r>
           <rPr>
@@ -194,7 +194,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CX3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000C000000}">
+    <comment ref="CW3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000C000000}">
       <text>
         <r>
           <rPr>
@@ -207,7 +207,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CY3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000D000000}">
+    <comment ref="CX3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000D000000}">
       <text>
         <r>
           <rPr>
@@ -220,7 +220,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CZ3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000E000000}">
+    <comment ref="CY3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000E000000}">
       <text>
         <r>
           <rPr>
@@ -233,7 +233,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="DA3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000F000000}">
+    <comment ref="CZ3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000F000000}">
       <text>
         <r>
           <rPr>
@@ -246,7 +246,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="DB3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000010000000}">
+    <comment ref="DA3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000010000000}">
       <text>
         <r>
           <rPr>
@@ -264,7 +264,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="536">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="671" uniqueCount="533">
   <si>
     <t>Bulkoad Sheet Instructions</t>
   </si>
@@ -398,9 +398,6 @@
     <t>ProductType</t>
   </si>
   <si>
-    <t>Style</t>
-  </si>
-  <si>
     <t>Pattern</t>
   </si>
   <si>
@@ -852,9 +849,6 @@
   </si>
   <si>
     <t>What type of product is this?</t>
-  </si>
-  <si>
-    <t>What is the style of this product? A style is the type of décor that this product is meant to match with.</t>
   </si>
   <si>
     <t>What is the pattern of the product? If there is more than one pattern, please select all that apply.</t>
@@ -991,9 +985,6 @@
   </si>
   <si>
     <t>Please choose from the following: Border; Tile; Roll; Wall Mural; Installation Tools; Double Roll; Adhesives &amp; Tools; Panel</t>
-  </si>
-  <si>
-    <t>Please choose from the following: Modern &amp; Contemporary; American Traditional; Traditional; Eclectic; Farmhouse / Country; Coastal; Rustic; Ornate Traditional; Tiffany; Industrial; Glam; Ornate Glam; Posh &amp; Luxe; Beachy; Nautical; Tropical; Cabin / Lodge; Mission/Shaker; Modern Rustic; Modern Farmhouse; French Country; Cottage Americana; Canadiana; Global Inspired; Bohemian; Sleek &amp; Chic Modern; Scandinavian; Mid-Century Modern; Bold &amp; Eclectic Modern; Retro; No Style; Children's; Vintage; Preppy; Modern; Casual; Garden; Classic; Country Rustic; Art Deco; Minimalist; Florentiner; Cabin; Contemporary; Country/Cottage; Mid-Century; French</t>
   </si>
   <si>
     <t>Please choose from the following: Abstract; Animal Print; Chevron; Damask; Floral; Geometric; Paisley; Plaid; Polka Dots; Striped; Toile; Brick; Solid Color; Stone; Wood &amp; Shiplap; Marble; Gingham; Camouflage; Ikat; Houndstooth; Patchwork; Ombre; Checkered; Argyle; No Pattern; Trellis; Dots; Starburst; Geometric Shapes; Irish Chain; Chevron / Zig Zag; Clear; Drunkard's Path; Moroccan; Oriental; Block Print; Arc; Vintage Look</t>
@@ -2420,6 +2411,9 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2427,9 +2421,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3473,7 +3464,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:DB780"/>
+  <dimension ref="A1:DA780"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="13" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="16.5" style="13" customWidth="1"/>
@@ -3513,10 +3504,10 @@
     <col min="55" max="59" width="16.33203125" style="19" customWidth="1"/>
     <col min="60" max="60" width="21.33203125" style="19" customWidth="1"/>
     <col min="61" max="61" width="24.33203125" style="19" customWidth="1"/>
-    <col min="62" max="106" width="24.33203125" customWidth="1"/>
+    <col min="62" max="105" width="24.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:106" hidden="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:105" hidden="1" x14ac:dyDescent="0.15">
       <c r="BI1" s="19" t="s">
         <v>43</v>
       </c>
@@ -3652,519 +3643,513 @@
       <c r="DA1" t="s">
         <v>87</v>
       </c>
-      <c r="DB1" t="s">
+    </row>
+    <row r="2" spans="1:105" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A2" s="9" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="2" spans="1:106" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="9" t="s">
+      <c r="B2" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="C2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="I2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="J2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="M2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="N2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="O2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="P2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="Q2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="R2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="S2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="T2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="U2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="V2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="W2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="X2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="Z2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="AA2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="AB2" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="AC2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="AD2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="AE2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="AF2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="AG2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="AH2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="AI2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="AJ2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="AK2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="AL2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="AM2" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="AN2" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AO2" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AP2" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AQ2" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AR2" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AS2" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AT2" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AU2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="AV2" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="AW2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="AX2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="AY2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="AZ2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="BA2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="BB2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="BC2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="BD2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="BE2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="BF2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="BG2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="BH2" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="BI2" s="55" t="s">
         <v>89</v>
       </c>
-      <c r="F2" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="I2" s="9" t="s">
+      <c r="BJ2" s="56" t="s">
+        <v>91</v>
+      </c>
+      <c r="BK2" s="56" t="s">
+        <v>91</v>
+      </c>
+      <c r="BL2" s="56" t="s">
+        <v>91</v>
+      </c>
+      <c r="BM2" s="57" t="s">
         <v>89</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="BN2" s="57" t="s">
         <v>89</v>
       </c>
-      <c r="K2" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="L2" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="M2" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="N2" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="O2" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="P2" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="Q2" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="R2" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="S2" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="T2" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="U2" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="V2" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="W2" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="X2" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="Y2" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="Z2" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="AA2" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="AB2" s="7" t="s">
+      <c r="BO2" s="56" t="s">
         <v>91</v>
       </c>
-      <c r="AC2" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="AD2" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="AE2" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="AF2" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="AG2" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="AH2" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="AI2" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="AJ2" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="AK2" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL2" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="AM2" s="7" t="s">
+      <c r="BP2" s="56" t="s">
         <v>91</v>
       </c>
-      <c r="AN2" s="7" t="s">
+      <c r="BQ2" s="56" t="s">
         <v>91</v>
       </c>
-      <c r="AO2" s="7" t="s">
+      <c r="BR2" s="56" t="s">
         <v>91</v>
-      </c>
-      <c r="AP2" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="AQ2" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="AR2" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="AS2" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="AT2" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="AU2" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="AV2" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="AW2" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="AX2" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="AY2" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="AZ2" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="BA2" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="BB2" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="BC2" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="BD2" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="BE2" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="BF2" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="BG2" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="BH2" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="BI2" s="55" t="s">
-        <v>90</v>
-      </c>
-      <c r="BJ2" s="56" t="s">
-        <v>92</v>
-      </c>
-      <c r="BK2" s="56" t="s">
-        <v>92</v>
-      </c>
-      <c r="BL2" s="56" t="s">
-        <v>92</v>
-      </c>
-      <c r="BM2" s="56" t="s">
-        <v>92</v>
-      </c>
-      <c r="BN2" s="57" t="s">
-        <v>90</v>
-      </c>
-      <c r="BO2" s="57" t="s">
-        <v>90</v>
-      </c>
-      <c r="BP2" s="56" t="s">
-        <v>92</v>
-      </c>
-      <c r="BQ2" s="56" t="s">
-        <v>92</v>
-      </c>
-      <c r="BR2" s="56" t="s">
-        <v>92</v>
       </c>
       <c r="BS2" s="56" t="s">
         <v>92</v>
       </c>
-      <c r="BT2" s="56" t="s">
-        <v>93</v>
+      <c r="BT2" s="57" t="s">
+        <v>89</v>
       </c>
       <c r="BU2" s="57" t="s">
+        <v>89</v>
+      </c>
+      <c r="BV2" s="56" t="s">
+        <v>91</v>
+      </c>
+      <c r="BW2" s="56" t="s">
+        <v>91</v>
+      </c>
+      <c r="BX2" s="56" t="s">
+        <v>91</v>
+      </c>
+      <c r="BY2" s="56" t="s">
+        <v>91</v>
+      </c>
+      <c r="BZ2" s="56" t="s">
+        <v>91</v>
+      </c>
+      <c r="CA2" s="56" t="s">
+        <v>91</v>
+      </c>
+      <c r="CB2" s="56" t="s">
+        <v>91</v>
+      </c>
+      <c r="CC2" s="56" t="s">
+        <v>91</v>
+      </c>
+      <c r="CD2" s="56" t="s">
+        <v>91</v>
+      </c>
+      <c r="CE2" s="57" t="s">
+        <v>89</v>
+      </c>
+      <c r="CF2" s="56" t="s">
+        <v>91</v>
+      </c>
+      <c r="CG2" s="56" t="s">
+        <v>91</v>
+      </c>
+      <c r="CH2" s="57" t="s">
+        <v>89</v>
+      </c>
+      <c r="CI2" s="57" t="s">
+        <v>89</v>
+      </c>
+      <c r="CJ2" s="57" t="s">
+        <v>89</v>
+      </c>
+      <c r="CK2" s="58" t="s">
         <v>90</v>
       </c>
-      <c r="BV2" s="57" t="s">
-        <v>90</v>
-      </c>
-      <c r="BW2" s="56" t="s">
-        <v>92</v>
-      </c>
-      <c r="BX2" s="56" t="s">
-        <v>92</v>
-      </c>
-      <c r="BY2" s="56" t="s">
-        <v>92</v>
-      </c>
-      <c r="BZ2" s="56" t="s">
-        <v>92</v>
-      </c>
-      <c r="CA2" s="56" t="s">
-        <v>92</v>
-      </c>
-      <c r="CB2" s="56" t="s">
-        <v>92</v>
-      </c>
-      <c r="CC2" s="56" t="s">
-        <v>92</v>
-      </c>
-      <c r="CD2" s="56" t="s">
-        <v>92</v>
-      </c>
-      <c r="CE2" s="56" t="s">
-        <v>92</v>
-      </c>
-      <c r="CF2" s="57" t="s">
-        <v>90</v>
-      </c>
-      <c r="CG2" s="56" t="s">
-        <v>92</v>
-      </c>
-      <c r="CH2" s="56" t="s">
-        <v>92</v>
-      </c>
-      <c r="CI2" s="57" t="s">
-        <v>90</v>
-      </c>
-      <c r="CJ2" s="57" t="s">
-        <v>90</v>
-      </c>
-      <c r="CK2" s="57" t="s">
-        <v>90</v>
-      </c>
-      <c r="CL2" s="58" t="s">
+      <c r="CL2" s="56" t="s">
         <v>91</v>
       </c>
       <c r="CM2" s="56" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="CN2" s="56" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="CO2" s="56" t="s">
         <v>92</v>
       </c>
       <c r="CP2" s="56" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="CQ2" s="56" t="s">
+        <v>91</v>
+      </c>
+      <c r="CR2" s="57" t="s">
+        <v>89</v>
+      </c>
+      <c r="CS2" s="57" t="s">
+        <v>89</v>
+      </c>
+      <c r="CT2" s="57" t="s">
+        <v>89</v>
+      </c>
+      <c r="CU2" s="56" t="s">
         <v>92</v>
       </c>
-      <c r="CR2" s="56" t="s">
-        <v>92</v>
-      </c>
-      <c r="CS2" s="57" t="s">
-        <v>90</v>
-      </c>
-      <c r="CT2" s="57" t="s">
-        <v>90</v>
-      </c>
-      <c r="CU2" s="57" t="s">
-        <v>90</v>
-      </c>
-      <c r="CV2" s="56" t="s">
-        <v>93</v>
-      </c>
-      <c r="CW2" s="57" t="s">
-        <v>90</v>
+      <c r="CV2" s="57" t="s">
+        <v>89</v>
+      </c>
+      <c r="CW2" s="56" t="s">
+        <v>91</v>
       </c>
       <c r="CX2" s="56" t="s">
         <v>92</v>
       </c>
       <c r="CY2" s="56" t="s">
+        <v>92</v>
+      </c>
+      <c r="CZ2" s="56" t="s">
+        <v>92</v>
+      </c>
+      <c r="DA2" s="56" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3" spans="1:105" ht="58.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A3" s="70" t="s">
         <v>93</v>
       </c>
-      <c r="CZ2" s="56" t="s">
-        <v>93</v>
-      </c>
-      <c r="DA2" s="56" t="s">
-        <v>93</v>
-      </c>
-      <c r="DB2" s="56" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="3" spans="1:106" ht="58.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="69" t="s">
+      <c r="B3" s="70" t="s">
         <v>94</v>
       </c>
-      <c r="B3" s="69" t="s">
+      <c r="C3" s="70" t="s">
         <v>95</v>
       </c>
-      <c r="C3" s="69" t="s">
+      <c r="D3" s="70" t="s">
         <v>96</v>
       </c>
-      <c r="D3" s="69" t="s">
+      <c r="E3" s="70" t="s">
         <v>97</v>
       </c>
-      <c r="E3" s="69" t="s">
+      <c r="F3" s="70" t="s">
         <v>98</v>
       </c>
-      <c r="F3" s="69" t="s">
+      <c r="G3" s="69" t="s">
         <v>99</v>
       </c>
-      <c r="G3" s="72" t="s">
+      <c r="H3" s="70" t="s">
         <v>100</v>
       </c>
-      <c r="H3" s="69" t="s">
+      <c r="I3" s="70" t="s">
         <v>101</v>
       </c>
-      <c r="I3" s="69" t="s">
+      <c r="J3" s="70" t="s">
         <v>102</v>
       </c>
-      <c r="J3" s="69" t="s">
+      <c r="K3" s="70" t="s">
         <v>103</v>
       </c>
-      <c r="K3" s="69" t="s">
+      <c r="L3" s="70" t="s">
         <v>104</v>
       </c>
-      <c r="L3" s="69" t="s">
+      <c r="M3" s="70" t="s">
         <v>105</v>
       </c>
-      <c r="M3" s="69" t="s">
+      <c r="N3" s="70" t="s">
         <v>106</v>
       </c>
-      <c r="N3" s="69" t="s">
+      <c r="O3" s="70" t="s">
         <v>107</v>
       </c>
-      <c r="O3" s="69" t="s">
+      <c r="P3" s="70" t="s">
         <v>108</v>
       </c>
-      <c r="P3" s="69" t="s">
+      <c r="Q3" s="70" t="s">
         <v>109</v>
       </c>
-      <c r="Q3" s="69" t="s">
+      <c r="R3" s="70" t="s">
         <v>110</v>
       </c>
-      <c r="R3" s="69" t="s">
+      <c r="S3" s="70" t="s">
         <v>111</v>
       </c>
-      <c r="S3" s="69" t="s">
+      <c r="T3" s="70" t="s">
         <v>112</v>
       </c>
-      <c r="T3" s="69" t="s">
+      <c r="U3" s="70" t="s">
         <v>113</v>
       </c>
-      <c r="U3" s="69" t="s">
+      <c r="V3" s="70" t="s">
         <v>114</v>
       </c>
-      <c r="V3" s="69" t="s">
+      <c r="W3" s="70" t="s">
         <v>115</v>
       </c>
-      <c r="W3" s="69" t="s">
+      <c r="X3" s="70" t="s">
         <v>116</v>
       </c>
-      <c r="X3" s="69" t="s">
+      <c r="Y3" s="70" t="s">
         <v>117</v>
       </c>
-      <c r="Y3" s="69" t="s">
+      <c r="Z3" s="70" t="s">
         <v>118</v>
       </c>
-      <c r="Z3" s="69" t="s">
+      <c r="AA3" s="70" t="s">
         <v>119</v>
       </c>
-      <c r="AA3" s="69" t="s">
+      <c r="AB3" s="70" t="s">
         <v>120</v>
       </c>
-      <c r="AB3" s="69" t="s">
+      <c r="AC3" s="70" t="s">
         <v>121</v>
       </c>
-      <c r="AC3" s="69" t="s">
+      <c r="AD3" s="70" t="s">
         <v>122</v>
       </c>
-      <c r="AD3" s="69" t="s">
+      <c r="AE3" s="70" t="s">
         <v>123</v>
       </c>
-      <c r="AE3" s="69" t="s">
+      <c r="AF3" s="70" t="s">
         <v>124</v>
       </c>
-      <c r="AF3" s="69" t="s">
+      <c r="AG3" s="70" t="s">
         <v>125</v>
       </c>
-      <c r="AG3" s="69" t="s">
+      <c r="AH3" s="70" t="s">
         <v>126</v>
       </c>
-      <c r="AH3" s="69" t="s">
+      <c r="AI3" s="70" t="s">
         <v>127</v>
       </c>
-      <c r="AI3" s="69" t="s">
+      <c r="AJ3" s="70" t="s">
         <v>128</v>
       </c>
-      <c r="AJ3" s="69" t="s">
+      <c r="AK3" s="70" t="s">
         <v>129</v>
       </c>
-      <c r="AK3" s="69" t="s">
+      <c r="AL3" s="70" t="s">
         <v>130</v>
       </c>
-      <c r="AL3" s="69" t="s">
+      <c r="AM3" s="70" t="s">
         <v>131</v>
       </c>
-      <c r="AM3" s="69" t="s">
+      <c r="AN3" s="70" t="s">
         <v>132</v>
       </c>
-      <c r="AN3" s="69" t="s">
+      <c r="AO3" s="70" t="s">
         <v>133</v>
       </c>
-      <c r="AO3" s="69" t="s">
+      <c r="AP3" s="70" t="s">
         <v>134</v>
       </c>
-      <c r="AP3" s="69" t="s">
+      <c r="AQ3" s="70" t="s">
         <v>135</v>
       </c>
-      <c r="AQ3" s="69" t="s">
+      <c r="AR3" s="70" t="s">
         <v>136</v>
       </c>
-      <c r="AR3" s="69" t="s">
+      <c r="AS3" s="70" t="s">
         <v>137</v>
       </c>
-      <c r="AS3" s="69" t="s">
+      <c r="AT3" s="70" t="s">
         <v>138</v>
       </c>
-      <c r="AT3" s="69" t="s">
+      <c r="AU3" s="70" t="s">
         <v>139</v>
       </c>
-      <c r="AU3" s="69" t="s">
+      <c r="AV3" s="70" t="s">
         <v>140</v>
       </c>
-      <c r="AV3" s="69" t="s">
+      <c r="AW3" s="70" t="s">
         <v>141</v>
       </c>
-      <c r="AW3" s="69" t="s">
+      <c r="AX3" s="70" t="s">
         <v>142</v>
       </c>
-      <c r="AX3" s="69" t="s">
+      <c r="AY3" s="69" t="s">
         <v>143</v>
       </c>
-      <c r="AY3" s="72" t="s">
+      <c r="AZ3" s="69" t="s">
         <v>144</v>
       </c>
-      <c r="AZ3" s="72" t="s">
+      <c r="BA3" s="69" t="s">
         <v>145</v>
       </c>
-      <c r="BA3" s="72" t="s">
+      <c r="BB3" s="70" t="s">
         <v>146</v>
       </c>
-      <c r="BB3" s="69" t="s">
+      <c r="BC3" s="70" t="s">
         <v>147</v>
       </c>
-      <c r="BC3" s="69" t="s">
+      <c r="BD3" s="70" t="s">
         <v>148</v>
       </c>
-      <c r="BD3" s="69" t="s">
+      <c r="BE3" s="70" t="s">
         <v>149</v>
       </c>
-      <c r="BE3" s="69" t="s">
+      <c r="BF3" s="70" t="s">
         <v>150</v>
       </c>
-      <c r="BF3" s="69" t="s">
+      <c r="BG3" s="70" t="s">
         <v>151</v>
       </c>
-      <c r="BG3" s="69" t="s">
+      <c r="BH3" s="70" t="s">
         <v>152</v>
       </c>
-      <c r="BH3" s="69" t="s">
+      <c r="BI3" s="59" t="s">
         <v>153</v>
-      </c>
-      <c r="BI3" s="59" t="s">
-        <v>154</v>
       </c>
       <c r="BJ3" s="56" t="s">
         <v>44</v>
       </c>
       <c r="BK3" s="56" t="s">
-        <v>45</v>
+        <v>154</v>
       </c>
       <c r="BL3" s="56" t="s">
         <v>155</v>
@@ -4199,10 +4184,10 @@
       <c r="BV3" s="56" t="s">
         <v>165</v>
       </c>
-      <c r="BW3" s="56" t="s">
+      <c r="BW3" s="60" t="s">
         <v>166</v>
       </c>
-      <c r="BX3" s="60" t="s">
+      <c r="BX3" s="61" t="s">
         <v>167</v>
       </c>
       <c r="BY3" s="61" t="s">
@@ -4211,52 +4196,52 @@
       <c r="BZ3" s="61" t="s">
         <v>169</v>
       </c>
-      <c r="CA3" s="61" t="s">
+      <c r="CA3" s="56" t="s">
+        <v>61</v>
+      </c>
+      <c r="CB3" s="56" t="s">
         <v>170</v>
       </c>
-      <c r="CB3" s="56" t="s">
-        <v>62</v>
-      </c>
       <c r="CC3" s="56" t="s">
+        <v>63</v>
+      </c>
+      <c r="CD3" s="56" t="s">
         <v>171</v>
       </c>
-      <c r="CD3" s="56" t="s">
-        <v>64</v>
-      </c>
       <c r="CE3" s="56" t="s">
+        <v>65</v>
+      </c>
+      <c r="CF3" s="60" t="s">
         <v>172</v>
       </c>
-      <c r="CF3" s="56" t="s">
-        <v>66</v>
-      </c>
-      <c r="CG3" s="60" t="s">
+      <c r="CG3" s="61" t="s">
         <v>173</v>
       </c>
-      <c r="CH3" s="61" t="s">
+      <c r="CH3" s="56" t="s">
         <v>174</v>
       </c>
       <c r="CI3" s="56" t="s">
         <v>175</v>
       </c>
-      <c r="CJ3" s="56" t="s">
+      <c r="CJ3" s="60" t="s">
         <v>176</v>
       </c>
-      <c r="CK3" s="60" t="s">
+      <c r="CK3" s="61" t="s">
         <v>177</v>
       </c>
-      <c r="CL3" s="61" t="s">
+      <c r="CL3" s="56" t="s">
         <v>178</v>
       </c>
       <c r="CM3" s="56" t="s">
         <v>179</v>
       </c>
-      <c r="CN3" s="56" t="s">
+      <c r="CN3" s="60" t="s">
         <v>180</v>
       </c>
-      <c r="CO3" s="60" t="s">
+      <c r="CO3" s="61" t="s">
         <v>181</v>
       </c>
-      <c r="CP3" s="61" t="s">
+      <c r="CP3" s="56" t="s">
         <v>182</v>
       </c>
       <c r="CQ3" s="56" t="s">
@@ -4274,16 +4259,16 @@
       <c r="CU3" s="56" t="s">
         <v>187</v>
       </c>
-      <c r="CV3" s="56" t="s">
+      <c r="CV3" s="60" t="s">
         <v>188</v>
       </c>
-      <c r="CW3" s="60" t="s">
+      <c r="CW3" s="61" t="s">
         <v>189</v>
       </c>
-      <c r="CX3" s="61" t="s">
+      <c r="CX3" s="60" t="s">
         <v>190</v>
       </c>
-      <c r="CY3" s="60" t="s">
+      <c r="CY3" s="61" t="s">
         <v>191</v>
       </c>
       <c r="CZ3" s="61" t="s">
@@ -4292,411 +4277,402 @@
       <c r="DA3" s="61" t="s">
         <v>193</v>
       </c>
-      <c r="DB3" s="61" t="s">
+    </row>
+    <row r="4" spans="1:105" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A4" s="71"/>
+      <c r="B4" s="71"/>
+      <c r="C4" s="71"/>
+      <c r="D4" s="71"/>
+      <c r="E4" s="71"/>
+      <c r="F4" s="71"/>
+      <c r="G4" s="69"/>
+      <c r="H4" s="71"/>
+      <c r="I4" s="71"/>
+      <c r="J4" s="71"/>
+      <c r="K4" s="71"/>
+      <c r="L4" s="71"/>
+      <c r="M4" s="71"/>
+      <c r="N4" s="71"/>
+      <c r="O4" s="71"/>
+      <c r="P4" s="71"/>
+      <c r="Q4" s="71"/>
+      <c r="R4" s="71"/>
+      <c r="S4" s="71"/>
+      <c r="T4" s="71"/>
+      <c r="U4" s="71"/>
+      <c r="V4" s="71"/>
+      <c r="W4" s="71"/>
+      <c r="X4" s="71"/>
+      <c r="Y4" s="71"/>
+      <c r="Z4" s="71"/>
+      <c r="AA4" s="71"/>
+      <c r="AB4" s="71"/>
+      <c r="AC4" s="71"/>
+      <c r="AD4" s="71"/>
+      <c r="AE4" s="71"/>
+      <c r="AF4" s="71"/>
+      <c r="AG4" s="71"/>
+      <c r="AH4" s="71"/>
+      <c r="AI4" s="71"/>
+      <c r="AJ4" s="71"/>
+      <c r="AK4" s="71"/>
+      <c r="AL4" s="71"/>
+      <c r="AM4" s="71"/>
+      <c r="AN4" s="71"/>
+      <c r="AO4" s="71"/>
+      <c r="AP4" s="71"/>
+      <c r="AQ4" s="71"/>
+      <c r="AR4" s="71"/>
+      <c r="AS4" s="71"/>
+      <c r="AT4" s="71"/>
+      <c r="AU4" s="71"/>
+      <c r="AV4" s="71"/>
+      <c r="AW4" s="71"/>
+      <c r="AX4" s="71"/>
+      <c r="AY4" s="69"/>
+      <c r="AZ4" s="69"/>
+      <c r="BA4" s="69"/>
+      <c r="BB4" s="71"/>
+      <c r="BC4" s="71"/>
+      <c r="BD4" s="71"/>
+      <c r="BE4" s="71"/>
+      <c r="BF4" s="71"/>
+      <c r="BG4" s="71"/>
+      <c r="BH4" s="71"/>
+      <c r="BI4" s="62" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="4" spans="1:106" ht="13" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="70"/>
-      <c r="B4" s="70"/>
-      <c r="C4" s="70"/>
-      <c r="D4" s="70"/>
-      <c r="E4" s="70"/>
-      <c r="F4" s="70"/>
-      <c r="G4" s="72"/>
-      <c r="H4" s="70"/>
-      <c r="I4" s="70"/>
-      <c r="J4" s="70"/>
-      <c r="K4" s="70"/>
-      <c r="L4" s="70"/>
-      <c r="M4" s="70"/>
-      <c r="N4" s="70"/>
-      <c r="O4" s="70"/>
-      <c r="P4" s="70"/>
-      <c r="Q4" s="70"/>
-      <c r="R4" s="70"/>
-      <c r="S4" s="70"/>
-      <c r="T4" s="70"/>
-      <c r="U4" s="70"/>
-      <c r="V4" s="70"/>
-      <c r="W4" s="70"/>
-      <c r="X4" s="70"/>
-      <c r="Y4" s="70"/>
-      <c r="Z4" s="70"/>
-      <c r="AA4" s="70"/>
-      <c r="AB4" s="70"/>
-      <c r="AC4" s="70"/>
-      <c r="AD4" s="70"/>
-      <c r="AE4" s="70"/>
-      <c r="AF4" s="70"/>
-      <c r="AG4" s="70"/>
-      <c r="AH4" s="70"/>
-      <c r="AI4" s="70"/>
-      <c r="AJ4" s="70"/>
-      <c r="AK4" s="70"/>
-      <c r="AL4" s="70"/>
-      <c r="AM4" s="70"/>
-      <c r="AN4" s="70"/>
-      <c r="AO4" s="70"/>
-      <c r="AP4" s="70"/>
-      <c r="AQ4" s="70"/>
-      <c r="AR4" s="70"/>
-      <c r="AS4" s="70"/>
-      <c r="AT4" s="70"/>
-      <c r="AU4" s="70"/>
-      <c r="AV4" s="70"/>
-      <c r="AW4" s="70"/>
-      <c r="AX4" s="70"/>
-      <c r="AY4" s="72"/>
-      <c r="AZ4" s="72"/>
-      <c r="BA4" s="72"/>
-      <c r="BB4" s="70"/>
-      <c r="BC4" s="70"/>
-      <c r="BD4" s="70"/>
-      <c r="BE4" s="70"/>
-      <c r="BF4" s="70"/>
-      <c r="BG4" s="70"/>
-      <c r="BH4" s="70"/>
-      <c r="BI4" s="62" t="s">
+      <c r="BJ4" s="63" t="s">
         <v>195</v>
       </c>
-      <c r="BJ4" s="63" t="s">
+      <c r="BK4" s="63" t="s">
         <v>196</v>
       </c>
-      <c r="BK4" s="63" t="s">
+      <c r="BL4" s="63" t="s">
         <v>197</v>
       </c>
-      <c r="BL4" s="63" t="s">
+      <c r="BM4" s="63" t="s">
         <v>198</v>
       </c>
-      <c r="BM4" s="63" t="s">
+      <c r="BN4" s="63" t="s">
         <v>199</v>
       </c>
-      <c r="BN4" s="63" t="s">
+      <c r="BO4" s="63" t="s">
         <v>200</v>
       </c>
-      <c r="BO4" s="63" t="s">
+      <c r="BP4" s="63" t="s">
         <v>201</v>
       </c>
-      <c r="BP4" s="63" t="s">
+      <c r="BQ4" s="63" t="s">
         <v>202</v>
       </c>
-      <c r="BQ4" s="63" t="s">
+      <c r="BR4" s="63" t="s">
         <v>203</v>
       </c>
-      <c r="BR4" s="63" t="s">
+      <c r="BS4" s="63" t="s">
         <v>204</v>
       </c>
-      <c r="BS4" s="63" t="s">
+      <c r="BT4" s="63" t="s">
         <v>205</v>
       </c>
-      <c r="BT4" s="63" t="s">
+      <c r="BU4" s="63" t="s">
         <v>206</v>
       </c>
-      <c r="BU4" s="63" t="s">
+      <c r="BV4" s="63" t="s">
         <v>207</v>
       </c>
-      <c r="BV4" s="63" t="s">
+      <c r="BW4" s="63" t="s">
         <v>208</v>
       </c>
-      <c r="BW4" s="63" t="s">
+      <c r="BX4" s="63" t="s">
         <v>209</v>
       </c>
-      <c r="BX4" s="63" t="s">
+      <c r="BY4" s="63" t="s">
         <v>210</v>
       </c>
-      <c r="BY4" s="63" t="s">
+      <c r="BZ4" s="63" t="s">
         <v>211</v>
       </c>
-      <c r="BZ4" s="63" t="s">
+      <c r="CA4" s="63" t="s">
         <v>212</v>
       </c>
-      <c r="CA4" s="63" t="s">
+      <c r="CB4" s="63" t="s">
         <v>213</v>
       </c>
-      <c r="CB4" s="63" t="s">
+      <c r="CC4" s="63" t="s">
         <v>214</v>
       </c>
-      <c r="CC4" s="63" t="s">
+      <c r="CD4" s="63" t="s">
         <v>215</v>
       </c>
-      <c r="CD4" s="63" t="s">
+      <c r="CE4" s="63" t="s">
         <v>216</v>
       </c>
-      <c r="CE4" s="63" t="s">
+      <c r="CF4" s="63" t="s">
         <v>217</v>
       </c>
-      <c r="CF4" s="63" t="s">
+      <c r="CG4" s="63" t="s">
         <v>218</v>
       </c>
-      <c r="CG4" s="63" t="s">
+      <c r="CH4" s="63" t="s">
         <v>219</v>
       </c>
-      <c r="CH4" s="63" t="s">
+      <c r="CI4" s="63" t="s">
         <v>220</v>
       </c>
-      <c r="CI4" s="63" t="s">
+      <c r="CJ4" s="63" t="s">
         <v>221</v>
       </c>
-      <c r="CJ4" s="63" t="s">
+      <c r="CK4" s="63" t="s">
         <v>222</v>
       </c>
-      <c r="CK4" s="63" t="s">
+      <c r="CL4" s="63" t="s">
         <v>223</v>
       </c>
-      <c r="CL4" s="63" t="s">
+      <c r="CM4" s="63" t="s">
         <v>224</v>
       </c>
-      <c r="CM4" s="63" t="s">
+      <c r="CN4" s="63" t="s">
         <v>225</v>
       </c>
-      <c r="CN4" s="63" t="s">
+      <c r="CO4" s="63" t="s">
         <v>226</v>
       </c>
-      <c r="CO4" s="63" t="s">
+      <c r="CP4" s="63" t="s">
         <v>227</v>
       </c>
-      <c r="CP4" s="63" t="s">
+      <c r="CQ4" s="63" t="s">
         <v>228</v>
       </c>
-      <c r="CQ4" s="63" t="s">
+      <c r="CR4" s="63" t="s">
         <v>229</v>
       </c>
-      <c r="CR4" s="63" t="s">
+      <c r="CS4" s="63" t="s">
         <v>230</v>
       </c>
-      <c r="CS4" s="63" t="s">
+      <c r="CT4" s="63" t="s">
         <v>231</v>
       </c>
-      <c r="CT4" s="63" t="s">
+      <c r="CU4" s="63" t="s">
         <v>232</v>
       </c>
-      <c r="CU4" s="63" t="s">
+      <c r="CV4" s="63" t="s">
         <v>233</v>
       </c>
-      <c r="CV4" s="63" t="s">
+      <c r="CW4" s="63" t="s">
         <v>234</v>
       </c>
-      <c r="CW4" s="63" t="s">
+      <c r="CX4" s="63" t="s">
         <v>235</v>
       </c>
-      <c r="CX4" s="63" t="s">
+      <c r="CY4" s="63" t="s">
         <v>236</v>
       </c>
-      <c r="CY4" s="63" t="s">
+      <c r="CZ4" s="63" t="s">
         <v>237</v>
       </c>
-      <c r="CZ4" s="63" t="s">
+      <c r="DA4" s="63" t="s">
         <v>238</v>
       </c>
-      <c r="DA4" s="63" t="s">
+    </row>
+    <row r="5" spans="1:105" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A5" s="72"/>
+      <c r="B5" s="72"/>
+      <c r="C5" s="72"/>
+      <c r="D5" s="72"/>
+      <c r="E5" s="72"/>
+      <c r="F5" s="72"/>
+      <c r="G5" s="69"/>
+      <c r="H5" s="72"/>
+      <c r="I5" s="72"/>
+      <c r="J5" s="72"/>
+      <c r="K5" s="72"/>
+      <c r="L5" s="72"/>
+      <c r="M5" s="72"/>
+      <c r="N5" s="72"/>
+      <c r="O5" s="72"/>
+      <c r="P5" s="72"/>
+      <c r="Q5" s="72"/>
+      <c r="R5" s="72"/>
+      <c r="S5" s="72"/>
+      <c r="T5" s="72"/>
+      <c r="U5" s="72"/>
+      <c r="V5" s="72"/>
+      <c r="W5" s="72"/>
+      <c r="X5" s="72"/>
+      <c r="Y5" s="72"/>
+      <c r="Z5" s="72"/>
+      <c r="AA5" s="72"/>
+      <c r="AB5" s="72"/>
+      <c r="AC5" s="72"/>
+      <c r="AD5" s="72"/>
+      <c r="AE5" s="72"/>
+      <c r="AF5" s="72"/>
+      <c r="AG5" s="72"/>
+      <c r="AH5" s="72"/>
+      <c r="AI5" s="72"/>
+      <c r="AJ5" s="72"/>
+      <c r="AK5" s="72"/>
+      <c r="AL5" s="72"/>
+      <c r="AM5" s="72"/>
+      <c r="AN5" s="72"/>
+      <c r="AO5" s="72"/>
+      <c r="AP5" s="72"/>
+      <c r="AQ5" s="72"/>
+      <c r="AR5" s="72"/>
+      <c r="AS5" s="72"/>
+      <c r="AT5" s="72"/>
+      <c r="AU5" s="72"/>
+      <c r="AV5" s="72"/>
+      <c r="AW5" s="72"/>
+      <c r="AX5" s="72"/>
+      <c r="AY5" s="69"/>
+      <c r="AZ5" s="69"/>
+      <c r="BA5" s="69"/>
+      <c r="BB5" s="72"/>
+      <c r="BC5" s="72"/>
+      <c r="BD5" s="72"/>
+      <c r="BE5" s="72"/>
+      <c r="BF5" s="72"/>
+      <c r="BG5" s="72"/>
+      <c r="BH5" s="72"/>
+      <c r="BI5" s="62" t="s">
         <v>239</v>
       </c>
-      <c r="DB4" s="63" t="s">
+      <c r="BJ5" s="63" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="5" spans="1:106" ht="13" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="71"/>
-      <c r="B5" s="71"/>
-      <c r="C5" s="71"/>
-      <c r="D5" s="71"/>
-      <c r="E5" s="71"/>
-      <c r="F5" s="71"/>
-      <c r="G5" s="72"/>
-      <c r="H5" s="71"/>
-      <c r="I5" s="71"/>
-      <c r="J5" s="71"/>
-      <c r="K5" s="71"/>
-      <c r="L5" s="71"/>
-      <c r="M5" s="71"/>
-      <c r="N5" s="71"/>
-      <c r="O5" s="71"/>
-      <c r="P5" s="71"/>
-      <c r="Q5" s="71"/>
-      <c r="R5" s="71"/>
-      <c r="S5" s="71"/>
-      <c r="T5" s="71"/>
-      <c r="U5" s="71"/>
-      <c r="V5" s="71"/>
-      <c r="W5" s="71"/>
-      <c r="X5" s="71"/>
-      <c r="Y5" s="71"/>
-      <c r="Z5" s="71"/>
-      <c r="AA5" s="71"/>
-      <c r="AB5" s="71"/>
-      <c r="AC5" s="71"/>
-      <c r="AD5" s="71"/>
-      <c r="AE5" s="71"/>
-      <c r="AF5" s="71"/>
-      <c r="AG5" s="71"/>
-      <c r="AH5" s="71"/>
-      <c r="AI5" s="71"/>
-      <c r="AJ5" s="71"/>
-      <c r="AK5" s="71"/>
-      <c r="AL5" s="71"/>
-      <c r="AM5" s="71"/>
-      <c r="AN5" s="71"/>
-      <c r="AO5" s="71"/>
-      <c r="AP5" s="71"/>
-      <c r="AQ5" s="71"/>
-      <c r="AR5" s="71"/>
-      <c r="AS5" s="71"/>
-      <c r="AT5" s="71"/>
-      <c r="AU5" s="71"/>
-      <c r="AV5" s="71"/>
-      <c r="AW5" s="71"/>
-      <c r="AX5" s="71"/>
-      <c r="AY5" s="72"/>
-      <c r="AZ5" s="72"/>
-      <c r="BA5" s="72"/>
-      <c r="BB5" s="71"/>
-      <c r="BC5" s="71"/>
-      <c r="BD5" s="71"/>
-      <c r="BE5" s="71"/>
-      <c r="BF5" s="71"/>
-      <c r="BG5" s="71"/>
-      <c r="BH5" s="71"/>
-      <c r="BI5" s="62" t="s">
+      <c r="BK5" s="63" t="s">
         <v>241</v>
       </c>
-      <c r="BJ5" s="63" t="s">
+      <c r="BL5" s="63" t="s">
         <v>242</v>
       </c>
-      <c r="BK5" s="63" t="s">
+      <c r="BM5" s="63" t="s">
         <v>243</v>
       </c>
-      <c r="BL5" s="63" t="s">
+      <c r="BN5" s="63" t="s">
         <v>244</v>
       </c>
-      <c r="BM5" s="63" t="s">
+      <c r="BO5" s="63" t="s">
         <v>245</v>
       </c>
-      <c r="BN5" s="63" t="s">
+      <c r="BP5" s="63" t="s">
         <v>246</v>
       </c>
-      <c r="BO5" s="63" t="s">
+      <c r="BQ5" s="63" t="s">
         <v>247</v>
       </c>
-      <c r="BP5" s="63" t="s">
+      <c r="BR5" s="63" t="s">
         <v>248</v>
       </c>
-      <c r="BQ5" s="63" t="s">
+      <c r="BS5" s="63" t="s">
         <v>249</v>
       </c>
-      <c r="BR5" s="63" t="s">
+      <c r="BT5" s="63" t="s">
         <v>250</v>
       </c>
-      <c r="BS5" s="63" t="s">
-        <v>251</v>
-      </c>
-      <c r="BT5" s="63" t="s">
-        <v>252</v>
-      </c>
       <c r="BU5" s="63" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="BV5" s="63" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="BW5" s="63" t="s">
         <v>251</v>
       </c>
       <c r="BX5" s="63" t="s">
+        <v>252</v>
+      </c>
+      <c r="BY5" s="63" t="s">
+        <v>253</v>
+      </c>
+      <c r="BZ5" s="63" t="s">
         <v>254</v>
       </c>
-      <c r="BY5" s="63" t="s">
+      <c r="CA5" s="63" t="s">
         <v>255</v>
       </c>
-      <c r="BZ5" s="63" t="s">
+      <c r="CB5" s="63" t="s">
         <v>256</v>
       </c>
-      <c r="CA5" s="63" t="s">
+      <c r="CC5" s="63" t="s">
         <v>257</v>
       </c>
-      <c r="CB5" s="63" t="s">
+      <c r="CD5" s="63" t="s">
         <v>258</v>
       </c>
-      <c r="CC5" s="63" t="s">
+      <c r="CE5" s="63" t="s">
         <v>259</v>
       </c>
-      <c r="CD5" s="63" t="s">
+      <c r="CF5" s="63" t="s">
         <v>260</v>
       </c>
-      <c r="CE5" s="63" t="s">
+      <c r="CG5" s="63" t="s">
         <v>261</v>
       </c>
-      <c r="CF5" s="63" t="s">
+      <c r="CH5" s="63" t="s">
         <v>262</v>
       </c>
-      <c r="CG5" s="63" t="s">
+      <c r="CI5" s="63" t="s">
+        <v>248</v>
+      </c>
+      <c r="CJ5" s="63" t="s">
+        <v>248</v>
+      </c>
+      <c r="CK5" s="63" t="s">
         <v>263</v>
       </c>
-      <c r="CH5" s="63" t="s">
+      <c r="CL5" s="63" t="s">
+        <v>248</v>
+      </c>
+      <c r="CM5" s="63" t="s">
         <v>264</v>
       </c>
-      <c r="CI5" s="63" t="s">
+      <c r="CN5" s="63" t="s">
+        <v>248</v>
+      </c>
+      <c r="CO5" s="63" t="s">
         <v>265</v>
       </c>
-      <c r="CJ5" s="63" t="s">
-        <v>251</v>
-      </c>
-      <c r="CK5" s="63" t="s">
-        <v>251</v>
-      </c>
-      <c r="CL5" s="63" t="s">
+      <c r="CP5" s="63" t="s">
+        <v>248</v>
+      </c>
+      <c r="CQ5" s="63" t="s">
         <v>266</v>
       </c>
-      <c r="CM5" s="63" t="s">
-        <v>251</v>
-      </c>
-      <c r="CN5" s="63" t="s">
+      <c r="CR5" s="63" t="s">
+        <v>261</v>
+      </c>
+      <c r="CS5" s="63" t="s">
+        <v>261</v>
+      </c>
+      <c r="CT5" s="63" t="s">
+        <v>261</v>
+      </c>
+      <c r="CU5" s="63" t="s">
+        <v>261</v>
+      </c>
+      <c r="CV5" s="63" t="s">
+        <v>248</v>
+      </c>
+      <c r="CW5" s="63" t="s">
         <v>267</v>
       </c>
-      <c r="CO5" s="63" t="s">
-        <v>251</v>
-      </c>
-      <c r="CP5" s="63" t="s">
+      <c r="CX5" s="63" t="s">
+        <v>248</v>
+      </c>
+      <c r="CY5" s="63" t="s">
         <v>268</v>
       </c>
-      <c r="CQ5" s="63" t="s">
-        <v>251</v>
-      </c>
-      <c r="CR5" s="63" t="s">
+      <c r="CZ5" s="63" t="s">
         <v>269</v>
       </c>
-      <c r="CS5" s="63" t="s">
-        <v>264</v>
-      </c>
-      <c r="CT5" s="63" t="s">
-        <v>264</v>
-      </c>
-      <c r="CU5" s="63" t="s">
-        <v>264</v>
-      </c>
-      <c r="CV5" s="63" t="s">
-        <v>264</v>
-      </c>
-      <c r="CW5" s="63" t="s">
-        <v>251</v>
-      </c>
-      <c r="CX5" s="63" t="s">
+      <c r="DA5" s="63" t="s">
         <v>270</v>
       </c>
-      <c r="CY5" s="63" t="s">
-        <v>251</v>
-      </c>
-      <c r="CZ5" s="63" t="s">
-        <v>271</v>
-      </c>
-      <c r="DA5" s="63" t="s">
-        <v>272</v>
-      </c>
-      <c r="DB5" s="63" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="6" spans="1:106" s="12" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="6" spans="1:105" s="12" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="10"/>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -4751,7 +4727,7 @@
       <c r="BA6" s="10"/>
       <c r="BB6" s="10"/>
     </row>
-    <row r="7" spans="1:106" s="12" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:105" s="12" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="10"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -4806,7 +4782,7 @@
       <c r="BA7" s="10"/>
       <c r="BB7" s="10"/>
     </row>
-    <row r="8" spans="1:106" s="12" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:105" s="12" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="10"/>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
@@ -4861,7 +4837,7 @@
       <c r="BA8" s="10"/>
       <c r="BB8" s="10"/>
     </row>
-    <row r="9" spans="1:106" s="12" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:105" s="12" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="10"/>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -4916,7 +4892,7 @@
       <c r="BA9" s="10"/>
       <c r="BB9" s="10"/>
     </row>
-    <row r="10" spans="1:106" s="12" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:105" s="12" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="10"/>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -4971,7 +4947,7 @@
       <c r="BA10" s="10"/>
       <c r="BB10" s="10"/>
     </row>
-    <row r="11" spans="1:106" s="12" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:105" s="12" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="10"/>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -5026,7 +5002,7 @@
       <c r="BA11" s="10"/>
       <c r="BB11" s="10"/>
     </row>
-    <row r="12" spans="1:106" s="12" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:105" s="12" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="10"/>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -5081,7 +5057,7 @@
       <c r="BA12" s="10"/>
       <c r="BB12" s="10"/>
     </row>
-    <row r="13" spans="1:106" s="12" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:105" s="12" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="10"/>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -5136,7 +5112,7 @@
       <c r="BA13" s="10"/>
       <c r="BB13" s="10"/>
     </row>
-    <row r="14" spans="1:106" s="12" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:105" s="12" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="10"/>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
@@ -5191,7 +5167,7 @@
       <c r="BA14" s="10"/>
       <c r="BB14" s="10"/>
     </row>
-    <row r="15" spans="1:106" s="12" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:105" s="12" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="10"/>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
@@ -5246,7 +5222,7 @@
       <c r="BA15" s="10"/>
       <c r="BB15" s="10"/>
     </row>
-    <row r="16" spans="1:106" s="12" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:105" s="12" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="10"/>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
@@ -47326,6 +47302,50 @@
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <autoFilter ref="A3:AX5" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <mergeCells count="60">
+    <mergeCell ref="F3:F5"/>
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="C3:C5"/>
+    <mergeCell ref="D3:D5"/>
+    <mergeCell ref="E3:E5"/>
+    <mergeCell ref="H3:H5"/>
+    <mergeCell ref="I3:I5"/>
+    <mergeCell ref="J3:J5"/>
+    <mergeCell ref="K3:K5"/>
+    <mergeCell ref="L3:L5"/>
+    <mergeCell ref="M3:M5"/>
+    <mergeCell ref="U3:U5"/>
+    <mergeCell ref="N3:N5"/>
+    <mergeCell ref="O3:O5"/>
+    <mergeCell ref="P3:P5"/>
+    <mergeCell ref="Q3:Q5"/>
+    <mergeCell ref="R3:R5"/>
+    <mergeCell ref="S3:S5"/>
+    <mergeCell ref="T3:T5"/>
+    <mergeCell ref="AG3:AG5"/>
+    <mergeCell ref="V3:V5"/>
+    <mergeCell ref="W3:W5"/>
+    <mergeCell ref="X3:X5"/>
+    <mergeCell ref="Y3:Y5"/>
+    <mergeCell ref="Z3:Z5"/>
+    <mergeCell ref="AA3:AA5"/>
+    <mergeCell ref="AB3:AB5"/>
+    <mergeCell ref="AC3:AC5"/>
+    <mergeCell ref="AD3:AD5"/>
+    <mergeCell ref="AE3:AE5"/>
+    <mergeCell ref="AF3:AF5"/>
+    <mergeCell ref="AS3:AS5"/>
+    <mergeCell ref="AH3:AH5"/>
+    <mergeCell ref="AI3:AI5"/>
+    <mergeCell ref="AJ3:AJ5"/>
+    <mergeCell ref="AK3:AK5"/>
+    <mergeCell ref="AL3:AL5"/>
+    <mergeCell ref="AM3:AM5"/>
+    <mergeCell ref="AN3:AN5"/>
+    <mergeCell ref="AO3:AO5"/>
+    <mergeCell ref="AP3:AP5"/>
+    <mergeCell ref="AQ3:AQ5"/>
+    <mergeCell ref="AR3:AR5"/>
     <mergeCell ref="G3:G5"/>
     <mergeCell ref="BH3:BH5"/>
     <mergeCell ref="BC3:BC5"/>
@@ -47342,50 +47362,6 @@
     <mergeCell ref="BE3:BE5"/>
     <mergeCell ref="BF3:BF5"/>
     <mergeCell ref="BG3:BG5"/>
-    <mergeCell ref="AS3:AS5"/>
-    <mergeCell ref="AH3:AH5"/>
-    <mergeCell ref="AI3:AI5"/>
-    <mergeCell ref="AJ3:AJ5"/>
-    <mergeCell ref="AK3:AK5"/>
-    <mergeCell ref="AL3:AL5"/>
-    <mergeCell ref="AM3:AM5"/>
-    <mergeCell ref="AN3:AN5"/>
-    <mergeCell ref="AO3:AO5"/>
-    <mergeCell ref="AP3:AP5"/>
-    <mergeCell ref="AQ3:AQ5"/>
-    <mergeCell ref="AR3:AR5"/>
-    <mergeCell ref="AG3:AG5"/>
-    <mergeCell ref="V3:V5"/>
-    <mergeCell ref="W3:W5"/>
-    <mergeCell ref="X3:X5"/>
-    <mergeCell ref="Y3:Y5"/>
-    <mergeCell ref="Z3:Z5"/>
-    <mergeCell ref="AA3:AA5"/>
-    <mergeCell ref="AB3:AB5"/>
-    <mergeCell ref="AC3:AC5"/>
-    <mergeCell ref="AD3:AD5"/>
-    <mergeCell ref="AE3:AE5"/>
-    <mergeCell ref="AF3:AF5"/>
-    <mergeCell ref="M3:M5"/>
-    <mergeCell ref="U3:U5"/>
-    <mergeCell ref="N3:N5"/>
-    <mergeCell ref="O3:O5"/>
-    <mergeCell ref="P3:P5"/>
-    <mergeCell ref="Q3:Q5"/>
-    <mergeCell ref="R3:R5"/>
-    <mergeCell ref="S3:S5"/>
-    <mergeCell ref="T3:T5"/>
-    <mergeCell ref="H3:H5"/>
-    <mergeCell ref="I3:I5"/>
-    <mergeCell ref="J3:J5"/>
-    <mergeCell ref="K3:K5"/>
-    <mergeCell ref="L3:L5"/>
-    <mergeCell ref="F3:F5"/>
-    <mergeCell ref="A3:A5"/>
-    <mergeCell ref="B3:B5"/>
-    <mergeCell ref="C3:C5"/>
-    <mergeCell ref="D3:D5"/>
-    <mergeCell ref="E3:E5"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B1048576">
     <cfRule type="expression" dxfId="23" priority="14">
@@ -47625,37 +47601,37 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A1" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F1"/>
     </row>
     <row r="2" spans="1:6" ht="26" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>274</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>275</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>276</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>277</v>
       </c>
       <c r="F2"/>
     </row>
@@ -47721,19 +47697,19 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A1" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C1"/>
     </row>
     <row r="2" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="C2"/>
     </row>
@@ -47765,20 +47741,20 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A1" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C1"/>
       <c r="D1"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A2" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="C2"/>
       <c r="D2"/>
@@ -47809,24 +47785,24 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A1" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="47" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
     </row>
   </sheetData>
@@ -47863,21 +47839,21 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A1" s="3" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A2" s="2" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="E2" s="1">
         <v>2</v>
@@ -47885,1259 +47861,1259 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A3" s="2" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A4" s="2" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A5" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A6" s="2" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.15">
       <c r="C7" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.15">
       <c r="C8" s="2" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.15">
       <c r="C9" s="2" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.15">
       <c r="C10" s="2" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.15">
       <c r="C11" s="2" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.15">
       <c r="C12" s="2" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.15">
       <c r="C13" s="2" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.15">
       <c r="C14" s="2" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.15">
       <c r="C15" s="2" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.15">
       <c r="C16" s="2" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
     </row>
     <row r="17" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C17" s="2" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
     </row>
     <row r="18" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C18" s="2" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
     </row>
     <row r="19" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C19" s="2" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
     </row>
     <row r="20" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C20" s="2" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
     </row>
     <row r="21" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C21" s="2" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
     </row>
     <row r="22" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C22" s="2" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="23" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C23" s="2" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
     </row>
     <row r="24" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C24" s="2" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
     </row>
     <row r="25" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C25" s="2" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="26" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C26" s="2" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
     </row>
     <row r="27" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C27" s="2" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
     </row>
     <row r="28" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C28" s="2" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
     </row>
     <row r="29" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C29" s="2" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
     </row>
     <row r="30" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C30" s="2" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
     </row>
     <row r="31" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C31" s="2" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
     </row>
     <row r="32" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C32" s="2" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
     </row>
     <row r="33" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C33" s="2" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
     </row>
     <row r="34" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C34" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
     </row>
     <row r="35" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C35" s="2" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
     </row>
     <row r="36" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C36" s="2" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
     </row>
     <row r="37" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C37" s="2" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
     </row>
     <row r="38" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C38" s="2" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
     <row r="39" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C39" s="2" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="40" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C40" s="2" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="41" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C41" s="2" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="42" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C42" s="2" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="43" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C43" s="2" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="44" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C44" s="2" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="45" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C45" s="2" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
     <row r="46" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C46" s="2" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
     </row>
     <row r="47" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C47" s="2" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
     </row>
     <row r="48" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C48" s="2" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
     </row>
     <row r="49" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C49" s="2" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
     </row>
     <row r="50" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C50" s="2" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
     </row>
     <row r="51" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C51" s="2" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
     </row>
     <row r="52" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C52" s="2" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
     </row>
     <row r="53" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C53" s="2" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
     </row>
     <row r="54" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C54" s="2" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
     </row>
     <row r="55" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C55" s="2" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
     </row>
     <row r="56" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C56" s="2" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
     </row>
     <row r="57" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C57" s="2" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
     </row>
     <row r="58" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C58" s="2" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
     </row>
     <row r="59" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C59" s="2" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
     </row>
     <row r="60" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C60" s="2" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
     </row>
     <row r="61" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C61" s="2" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
     </row>
     <row r="62" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C62" s="2" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
     </row>
     <row r="63" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C63" s="2" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
     </row>
     <row r="64" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C64" s="2" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
     </row>
     <row r="65" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C65" s="2" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
     </row>
     <row r="66" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C66" s="2" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
     </row>
     <row r="67" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C67" s="2" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
     </row>
     <row r="68" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C68" s="2" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="69" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C69" s="2" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
     </row>
     <row r="70" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C70" s="2" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
     </row>
     <row r="71" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C71" s="2" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
     </row>
     <row r="72" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C72" s="2" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
     </row>
     <row r="73" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C73" s="2" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
     </row>
     <row r="74" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C74" s="2" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
     </row>
     <row r="75" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C75" s="2" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
     </row>
     <row r="76" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C76" s="2" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
     </row>
     <row r="77" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C77" s="2" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
     </row>
     <row r="78" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C78" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
     </row>
     <row r="79" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C79" s="2" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
     </row>
     <row r="80" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C80" s="2" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
     </row>
     <row r="81" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C81" s="2" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
     </row>
     <row r="82" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C82" s="2" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
     </row>
     <row r="83" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C83" s="2" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
     </row>
     <row r="84" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C84" s="2" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
     </row>
     <row r="85" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C85" s="2" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
     </row>
     <row r="86" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C86" s="2" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
     </row>
     <row r="87" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C87" s="2" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
     </row>
     <row r="88" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C88" s="2" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="89" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C89" s="2" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
     </row>
     <row r="90" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C90" s="2" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
     </row>
     <row r="91" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C91" s="2" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
     </row>
     <row r="92" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C92" s="2" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
     </row>
     <row r="93" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C93" s="2" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
     </row>
     <row r="94" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C94" s="2" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
     </row>
     <row r="95" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C95" s="2" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
     </row>
     <row r="96" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C96" s="2" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
     </row>
     <row r="97" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C97" s="2" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
     </row>
     <row r="98" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C98" s="2" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
     </row>
     <row r="99" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C99" s="2" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
     </row>
     <row r="100" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C100" s="2" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
     </row>
     <row r="101" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C101" s="2" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
     </row>
     <row r="102" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C102" s="2" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
     </row>
     <row r="103" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C103" s="2" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
     </row>
     <row r="104" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C104" s="2" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
     </row>
     <row r="105" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C105" s="2" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
     </row>
     <row r="106" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C106" s="2" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
     </row>
     <row r="107" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C107" s="2" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
     </row>
     <row r="108" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C108" s="2" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
     </row>
     <row r="109" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C109" s="2" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
     </row>
     <row r="110" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C110" s="2" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
     </row>
     <row r="111" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C111" s="2" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
     </row>
     <row r="112" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C112" s="2" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
     </row>
     <row r="113" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C113" s="2" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
     </row>
     <row r="114" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C114" s="2" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
     </row>
     <row r="115" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C115" s="2" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
     </row>
     <row r="116" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C116" s="2" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
     </row>
     <row r="117" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C117" s="2" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
     </row>
     <row r="118" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C118" s="2" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
     </row>
     <row r="119" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C119" s="2" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
     </row>
     <row r="120" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C120" s="2" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
     </row>
     <row r="121" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C121" s="2" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
     </row>
     <row r="122" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C122" s="2" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
     </row>
     <row r="123" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C123" s="2" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
     </row>
     <row r="124" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C124" s="2" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="125" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C125" s="2" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
     </row>
     <row r="126" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C126" s="2" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
     </row>
     <row r="127" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C127" s="2" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
     </row>
     <row r="128" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C128" s="2" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
     </row>
     <row r="129" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C129" s="2" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="130" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C130" s="2" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
     </row>
     <row r="131" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C131" s="2" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
     </row>
     <row r="132" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C132" s="2" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
     </row>
     <row r="133" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C133" s="2" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
     </row>
     <row r="134" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C134" s="2" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
     </row>
     <row r="135" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C135" s="2" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
     </row>
     <row r="136" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C136" s="2" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
     </row>
     <row r="137" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C137" s="2" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
     </row>
     <row r="138" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C138" s="2" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
     </row>
     <row r="139" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C139" s="2" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
     </row>
     <row r="140" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C140" s="2" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
     </row>
     <row r="141" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C141" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
     </row>
     <row r="142" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C142" s="2" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
     </row>
     <row r="143" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C143" s="2" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
     </row>
     <row r="144" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C144" s="2" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
     </row>
     <row r="145" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C145" s="2" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
     </row>
     <row r="146" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C146" s="2" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
     </row>
     <row r="147" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C147" s="2" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
     </row>
     <row r="148" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C148" s="2" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
     </row>
     <row r="149" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C149" s="2" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
     </row>
     <row r="150" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C150" s="2" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
     </row>
     <row r="151" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C151" s="2" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
     </row>
     <row r="152" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C152" s="2" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
     </row>
     <row r="153" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C153" s="2" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
     </row>
     <row r="154" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C154" s="2" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
     </row>
     <row r="155" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C155" s="2" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
     </row>
     <row r="156" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C156" s="2" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="157" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C157" s="2" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
     </row>
     <row r="158" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C158" s="2" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
     </row>
     <row r="159" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C159" s="2" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
     <row r="160" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C160" s="2" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
     </row>
     <row r="161" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C161" s="2" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
     </row>
     <row r="162" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C162" s="2" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
     <row r="163" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C163" s="2" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
     </row>
     <row r="164" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C164" s="2" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
     </row>
     <row r="165" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C165" s="2" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
     </row>
     <row r="166" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C166" s="2" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
     </row>
     <row r="167" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C167" s="2" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
     </row>
     <row r="168" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C168" s="2" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
     </row>
     <row r="169" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C169" s="2" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
     </row>
     <row r="170" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C170" s="2" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
     </row>
     <row r="171" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C171" s="2" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
     </row>
     <row r="172" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C172" s="2" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
     </row>
     <row r="173" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C173" s="2" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
     </row>
     <row r="174" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C174" s="2" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
     </row>
     <row r="175" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C175" s="2" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
     </row>
     <row r="176" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C176" s="2" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
     </row>
     <row r="177" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C177" s="2" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
     </row>
     <row r="178" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C178" s="2" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
     </row>
     <row r="179" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C179" s="2" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
     </row>
     <row r="180" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C180" s="2" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
     </row>
     <row r="181" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C181" s="2" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
     </row>
     <row r="182" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C182" s="2" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
     </row>
     <row r="183" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C183" s="2" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
     </row>
     <row r="184" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C184" s="2" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
     </row>
     <row r="185" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C185" s="2" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
     </row>
     <row r="186" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C186" s="2" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
     </row>
     <row r="187" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C187" s="2" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
     </row>
     <row r="188" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C188" s="2" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
     </row>
     <row r="189" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C189" s="2" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
     </row>
     <row r="190" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C190" s="2" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
     </row>
     <row r="191" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C191" s="2" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
     </row>
     <row r="192" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C192" s="2" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
     </row>
     <row r="193" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C193" s="2" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
     </row>
     <row r="194" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C194" s="2" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
     </row>
     <row r="195" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C195" s="2" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
     </row>
     <row r="196" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C196" s="2" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
     </row>
     <row r="197" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C197" s="2" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
     </row>
     <row r="198" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C198" s="2" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
     </row>
     <row r="199" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C199" s="2" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
     </row>
     <row r="200" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C200" s="2" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
     </row>
     <row r="201" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C201" s="2" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
     </row>
     <row r="202" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C202" s="2" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
     </row>
     <row r="203" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C203" s="2" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
     </row>
     <row r="204" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C204" s="2" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
     </row>
     <row r="205" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C205" s="2" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
     </row>
     <row r="206" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C206" s="2" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
     </row>
     <row r="207" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C207" s="2" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
     </row>
     <row r="208" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C208" s="2" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
     </row>
     <row r="209" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C209" s="2" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
     </row>
     <row r="210" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C210" s="2" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
     </row>
     <row r="211" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C211" s="2" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
     </row>
     <row r="212" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C212" s="2" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
     </row>
     <row r="213" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C213" s="2" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
     </row>
     <row r="214" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C214" s="2" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
     </row>
     <row r="215" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C215" s="2" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
     </row>
     <row r="216" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C216" s="2" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
     </row>
     <row r="217" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C217" s="2" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
     </row>
     <row r="218" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C218" s="2" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
     </row>
     <row r="219" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C219" s="2" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
     </row>
     <row r="220" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C220" s="2" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
     </row>
     <row r="221" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C221" s="2" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
     </row>
     <row r="222" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C222" s="2" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
     </row>
     <row r="223" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C223" s="2" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
     </row>
     <row r="224" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C224" s="2" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
     </row>
     <row r="225" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C225" s="2" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
     </row>
     <row r="226" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C226" s="2" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
     </row>
     <row r="227" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C227" s="2" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
     </row>
     <row r="228" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C228" s="2" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
     </row>
     <row r="229" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C229" s="2" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
     </row>
     <row r="230" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C230" s="2" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
     </row>
     <row r="231" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C231" s="2" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
     </row>
     <row r="232" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C232" s="2" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
     </row>
     <row r="233" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C233" s="2" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
     </row>
     <row r="234" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C234" s="2" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
     </row>
     <row r="235" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C235" s="2" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
     </row>
     <row r="236" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C236" s="2" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
     </row>
     <row r="237" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C237" s="2" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
     </row>
     <row r="238" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C238" s="2" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
     </row>
     <row r="239" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C239" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
     </row>
     <row r="240" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C240" s="2" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
     </row>
     <row r="241" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C241" s="2" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
     </row>
     <row r="242" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C242" s="2" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
     </row>
     <row r="243" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C243" s="2" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
     </row>
     <row r="244" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C244" s="2" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
     </row>
     <row r="245" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C245" s="2" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
     </row>
     <row r="246" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C246" s="2" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
     </row>
     <row r="247" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C247" s="2" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
     </row>
     <row r="248" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C248" s="2" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
     </row>
     <row r="249" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C249" s="2" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
     </row>
     <row r="250" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C250" s="2" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
     </row>
     <row r="251" spans="3:3" x14ac:dyDescent="0.15">
       <c r="C251" s="2" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
     </row>
   </sheetData>

</xml_diff>